<commit_message>
Fixed issue when sorting ranges with blank cells.
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Ranges/SortExample.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Ranges/SortExample.xlsx
@@ -580,6 +580,8 @@
       <x:c r="C3" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="D3" s="0" t="s"/>
+      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -598,6 +600,8 @@
       <x:c r="C4" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D4" s="0" t="s"/>
+      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -616,6 +620,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s"/>
+      <x:c r="D5" s="0" t="s"/>
+      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -636,6 +642,8 @@
       <x:c r="C6" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D6" s="0" t="s"/>
+      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -656,6 +664,8 @@
       <x:c r="C7" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="D7" s="0" t="s"/>
+      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="8" t="s"/>
       <x:c r="G7" s="8" t="s">
         <x:v>7</x:v>
@@ -672,6 +682,8 @@
       <x:c r="C8" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D8" s="0" t="s"/>
+      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -690,6 +702,8 @@
       <x:c r="C9" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="D9" s="0" t="s"/>
+      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -708,6 +722,8 @@
       <x:c r="C10" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D10" s="0" t="s"/>
+      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -970,6 +986,8 @@
       <x:c r="C5" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D5" s="0" t="s"/>
+      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="8" t="s"/>
       <x:c r="G5" s="8" t="s">
         <x:v>7</x:v>
@@ -986,6 +1004,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s"/>
+      <x:c r="D6" s="0" t="s"/>
+      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1006,6 +1026,8 @@
       <x:c r="C7" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D7" s="0" t="s"/>
+      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1026,6 +1048,8 @@
       <x:c r="C8" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="D8" s="0" t="s"/>
+      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1044,6 +1068,8 @@
       <x:c r="C9" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D9" s="0" t="s"/>
+      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1064,6 +1090,8 @@
       <x:c r="C10" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="D10" s="0" t="s"/>
+      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1082,6 +1110,8 @@
       <x:c r="C11" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D11" s="0" t="s"/>
+      <x:c r="E11" s="0" t="s"/>
       <x:c r="F11" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1098,6 +1128,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s"/>
+      <x:c r="D12" s="0" t="s"/>
+      <x:c r="E12" s="0" t="s"/>
       <x:c r="F12" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1143,6 +1175,8 @@
       <x:c r="C3" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D3" s="0" t="s"/>
+      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1159,6 +1193,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s"/>
+      <x:c r="D4" s="0" t="s"/>
+      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1177,6 +1213,8 @@
       <x:c r="C5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D5" s="0" t="s"/>
+      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1197,6 +1235,8 @@
       <x:c r="C6" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="D6" s="0" t="s"/>
+      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="8" t="s"/>
       <x:c r="G6" s="8" t="s">
         <x:v>7</x:v>
@@ -1213,6 +1253,8 @@
       <x:c r="C7" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D7" s="0" t="s"/>
+      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1233,6 +1275,8 @@
       <x:c r="C8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="D8" s="0" t="s"/>
+      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1253,6 +1297,8 @@
       <x:c r="C9" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D9" s="0" t="s"/>
+      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1271,6 +1317,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="9" t="s"/>
+      <x:c r="D10" s="0" t="s"/>
+      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1312,6 +1360,8 @@
       <x:c r="A3" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="B3" s="0" t="s"/>
+      <x:c r="C3" s="0" t="s"/>
       <x:c r="D3" s="9" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -1320,6 +1370,8 @@
       <x:c r="A4" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="B4" s="0" t="s"/>
+      <x:c r="C4" s="0" t="s"/>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1328,18 +1380,24 @@
       <x:c r="A5" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="B5" s="0" t="s"/>
+      <x:c r="C5" s="0" t="s"/>
       <x:c r="D5" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="5" t="s"/>
+      <x:c r="B6" s="0" t="s"/>
+      <x:c r="C6" s="0" t="s"/>
       <x:c r="D6" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="8" t="s"/>
+      <x:c r="B7" s="0" t="s"/>
+      <x:c r="C7" s="0" t="s"/>
       <x:c r="D7" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1348,6 +1406,8 @@
       <x:c r="A8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="B8" s="0" t="s"/>
+      <x:c r="C8" s="0" t="s"/>
       <x:c r="D8" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1356,12 +1416,16 @@
       <x:c r="A9" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="B9" s="0" t="s"/>
+      <x:c r="C9" s="0" t="s"/>
       <x:c r="D9" s="8" t="s"/>
     </x:row>
     <x:row r="10" spans="1:4">
       <x:c r="A10" s="9" t="s">
         <x:v>14</x:v>
       </x:c>
+      <x:c r="B10" s="0" t="s"/>
+      <x:c r="C10" s="0" t="s"/>
       <x:c r="D10" s="5" t="s"/>
     </x:row>
   </x:sheetData>
@@ -1401,6 +1465,8 @@
       <x:c r="C3" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D3" s="0" t="s"/>
+      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1419,6 +1485,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s"/>
+      <x:c r="D4" s="0" t="s"/>
+      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1439,6 +1507,8 @@
       <x:c r="C5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D5" s="0" t="s"/>
+      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1459,6 +1529,8 @@
       <x:c r="C6" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="D6" s="0" t="s"/>
+      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1475,6 +1547,8 @@
       <x:c r="C7" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D7" s="0" t="s"/>
+      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1495,6 +1569,8 @@
       <x:c r="C8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="D8" s="0" t="s"/>
+      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1513,6 +1589,8 @@
       <x:c r="C9" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D9" s="0" t="s"/>
+      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1529,6 +1607,8 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="9" t="s"/>
+      <x:c r="D10" s="0" t="s"/>
+      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="8" t="s"/>
       <x:c r="G10" s="8" t="s">
         <x:v>7</x:v>

</xml_diff>

<commit_message>
Improved performance of previous fix.
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Ranges/SortExample.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Ranges/SortExample.xlsx
@@ -580,8 +580,6 @@
       <x:c r="C3" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s"/>
-      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -600,8 +598,6 @@
       <x:c r="C4" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s"/>
-      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -620,8 +616,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s"/>
-      <x:c r="D5" s="0" t="s"/>
-      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -642,8 +636,6 @@
       <x:c r="C6" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s"/>
-      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -664,8 +656,6 @@
       <x:c r="C7" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s"/>
-      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="8" t="s"/>
       <x:c r="G7" s="8" t="s">
         <x:v>7</x:v>
@@ -682,8 +672,6 @@
       <x:c r="C8" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s"/>
-      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -702,8 +690,6 @@
       <x:c r="C9" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s"/>
-      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -722,8 +708,6 @@
       <x:c r="C10" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D10" s="0" t="s"/>
-      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -986,8 +970,6 @@
       <x:c r="C5" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s"/>
-      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="8" t="s"/>
       <x:c r="G5" s="8" t="s">
         <x:v>7</x:v>
@@ -1004,8 +986,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="4" t="s"/>
-      <x:c r="D6" s="0" t="s"/>
-      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1026,8 +1006,6 @@
       <x:c r="C7" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s"/>
-      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1048,8 +1026,6 @@
       <x:c r="C8" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s"/>
-      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1068,8 +1044,6 @@
       <x:c r="C9" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s"/>
-      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1090,8 +1064,6 @@
       <x:c r="C10" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D10" s="0" t="s"/>
-      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1110,8 +1082,6 @@
       <x:c r="C11" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D11" s="0" t="s"/>
-      <x:c r="E11" s="0" t="s"/>
       <x:c r="F11" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1128,8 +1098,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s"/>
-      <x:c r="D12" s="0" t="s"/>
-      <x:c r="E12" s="0" t="s"/>
       <x:c r="F12" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1175,8 +1143,6 @@
       <x:c r="C3" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s"/>
-      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1193,8 +1159,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s"/>
-      <x:c r="D4" s="0" t="s"/>
-      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1213,8 +1177,6 @@
       <x:c r="C5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s"/>
-      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1235,8 +1197,6 @@
       <x:c r="C6" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s"/>
-      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="8" t="s"/>
       <x:c r="G6" s="8" t="s">
         <x:v>7</x:v>
@@ -1253,8 +1213,6 @@
       <x:c r="C7" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s"/>
-      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1275,8 +1233,6 @@
       <x:c r="C8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s"/>
-      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1297,8 +1253,6 @@
       <x:c r="C9" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s"/>
-      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1317,8 +1271,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="9" t="s"/>
-      <x:c r="D10" s="0" t="s"/>
-      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1360,8 +1312,6 @@
       <x:c r="A3" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s"/>
-      <x:c r="C3" s="0" t="s"/>
       <x:c r="D3" s="9" t="s">
         <x:v>14</x:v>
       </x:c>
@@ -1370,8 +1320,6 @@
       <x:c r="A4" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s"/>
-      <x:c r="C4" s="0" t="s"/>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1380,24 +1328,18 @@
       <x:c r="A5" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s"/>
-      <x:c r="C5" s="0" t="s"/>
       <x:c r="D5" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="5" t="s"/>
-      <x:c r="B6" s="0" t="s"/>
-      <x:c r="C6" s="0" t="s"/>
       <x:c r="D6" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="8" t="s"/>
-      <x:c r="B7" s="0" t="s"/>
-      <x:c r="C7" s="0" t="s"/>
       <x:c r="D7" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1406,8 +1348,6 @@
       <x:c r="A8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s"/>
-      <x:c r="C8" s="0" t="s"/>
       <x:c r="D8" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1416,16 +1356,12 @@
       <x:c r="A9" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s"/>
-      <x:c r="C9" s="0" t="s"/>
       <x:c r="D9" s="8" t="s"/>
     </x:row>
     <x:row r="10" spans="1:4">
       <x:c r="A10" s="9" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s"/>
-      <x:c r="C10" s="0" t="s"/>
       <x:c r="D10" s="5" t="s"/>
     </x:row>
   </x:sheetData>
@@ -1465,8 +1401,6 @@
       <x:c r="C3" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s"/>
-      <x:c r="E3" s="0" t="s"/>
       <x:c r="F3" s="7" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1485,8 +1419,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s"/>
-      <x:c r="D4" s="0" t="s"/>
-      <x:c r="E4" s="0" t="s"/>
       <x:c r="F4" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1507,8 +1439,6 @@
       <x:c r="C5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s"/>
-      <x:c r="E5" s="0" t="s"/>
       <x:c r="F5" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1529,8 +1459,6 @@
       <x:c r="C6" s="5" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s"/>
-      <x:c r="E6" s="0" t="s"/>
       <x:c r="F6" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
@@ -1547,8 +1475,6 @@
       <x:c r="C7" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s"/>
-      <x:c r="E7" s="0" t="s"/>
       <x:c r="F7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1569,8 +1495,6 @@
       <x:c r="C8" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s"/>
-      <x:c r="E8" s="0" t="s"/>
       <x:c r="F8" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1589,8 +1513,6 @@
       <x:c r="C9" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s"/>
-      <x:c r="E9" s="0" t="s"/>
       <x:c r="F9" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
@@ -1607,8 +1529,6 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="9" t="s"/>
-      <x:c r="D10" s="0" t="s"/>
-      <x:c r="E10" s="0" t="s"/>
       <x:c r="F10" s="8" t="s"/>
       <x:c r="G10" s="8" t="s">
         <x:v>7</x:v>

</xml_diff>